<commit_message>
feat(segmentation): enhance behavioral intelligence with category ratios
- replace top category flags with category ratio features (cat_ratio_*)
- introduce category grouping (fashion / accessory / other)
- improve behavioral signals in clustering (category mix, specialization)
- retain value + profit + risk features (RFM + returns)

segmentation now captures both value and behavior:
who is valuable + how they shop"
</commit_message>
<xml_diff>
--- a/reports/cluster_summary.xlsx
+++ b/reports/cluster_summary.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t xml:space="preserve">cluster</t>
   </si>
@@ -38,15 +38,9 @@
     <t xml:space="preserve">avg_basket</t>
   </si>
   <si>
-    <t xml:space="preserve">avg_price_level</t>
-  </si>
-  <si>
     <t xml:space="preserve">avg_weekend_ratio</t>
   </si>
   <si>
-    <t xml:space="preserve">avg_weekend_shopper</t>
-  </si>
-  <si>
     <t xml:space="preserve">avg_return_ratio</t>
   </si>
   <si>
@@ -65,13 +59,13 @@
     <t xml:space="preserve">avg_premium_ratio</t>
   </si>
   <si>
-    <t xml:space="preserve">topcat_fashion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">topcat_accessory</t>
-  </si>
-  <si>
-    <t xml:space="preserve">topcat_other</t>
+    <t xml:space="preserve">cat_ratio_accessory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cat_ratio_fashion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cat_ratio_other</t>
   </si>
 </sst>
 </file>
@@ -455,135 +449,117 @@
       <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
-        <v>18</v>
-      </c>
-      <c r="T1" t="s">
-        <v>19</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>2799</v>
+        <v>1725</v>
       </c>
       <c r="C2" t="n">
-        <v>4.39264022865309</v>
+        <v>5.60927536231884</v>
       </c>
       <c r="D2" t="n">
-        <v>13001.681850661</v>
+        <v>18373.4746086957</v>
       </c>
       <c r="E2" t="n">
-        <v>5859.09624866024</v>
+        <v>8543.12655072464</v>
       </c>
       <c r="F2" t="n">
-        <v>148.4880314398</v>
+        <v>105.241739130435</v>
       </c>
       <c r="G2" t="n">
-        <v>2.93676312968917</v>
+        <v>2.96811594202899</v>
       </c>
       <c r="H2" t="n">
-        <v>1300.13208398434</v>
-      </c>
-      <c r="I2" t="e">
-        <v>#NUM!</v>
+        <v>1432.23736506817</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.248524153896794</v>
       </c>
       <c r="J2" t="n">
-        <v>0.273982435778847</v>
+        <v>0.0395678587138224</v>
       </c>
       <c r="K2" t="n">
-        <v>0.157913540550196</v>
+        <v>0.0617396857524615</v>
       </c>
       <c r="L2" t="n">
-        <v>0.0463136337544607</v>
+        <v>0.465445433491757</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0785356699842196</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0.445838128329692</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0.526337341024595</v>
-      </c>
-      <c r="P2" t="e">
-        <v>#NUM!</v>
-      </c>
-      <c r="Q2" t="e">
-        <v>#NUM!</v>
+        <v>0.495621982510598</v>
+      </c>
+      <c r="N2" t="e">
+        <v>#NUM!</v>
+      </c>
+      <c r="O2" t="e">
+        <v>#NUM!</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.278111981166262</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.442871726047295</v>
       </c>
       <c r="R2" t="n">
-        <v>0.999285459092533</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0.000714540907466952</v>
-      </c>
-      <c r="T2" t="n">
-        <v>0</v>
+        <v>0.279016292786444</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>938</v>
+        <v>2829</v>
       </c>
       <c r="C3" t="n">
-        <v>4.06076759061834</v>
+        <v>3.52244609402616</v>
       </c>
       <c r="D3" t="n">
-        <v>10682.4320895522</v>
+        <v>8348.80445387063</v>
       </c>
       <c r="E3" t="n">
-        <v>4934.53251599147</v>
+        <v>3621.76323789325</v>
       </c>
       <c r="F3" t="n">
-        <v>153.575692963753</v>
+        <v>179.465182043125</v>
       </c>
       <c r="G3" t="n">
-        <v>2.86780383795309</v>
+        <v>2.95510781194768</v>
       </c>
       <c r="H3" t="n">
-        <v>1180.3736896093</v>
-      </c>
-      <c r="I3" t="e">
-        <v>#NUM!</v>
+        <v>1115.29746891481</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.175157792544418</v>
       </c>
       <c r="J3" t="n">
-        <v>0.274394283379376</v>
+        <v>0.0542352651317205</v>
       </c>
       <c r="K3" t="n">
-        <v>0.173773987206823</v>
+        <v>0.0955490741205182</v>
       </c>
       <c r="L3" t="n">
-        <v>0.0457328585759096</v>
+        <v>0.432928226828239</v>
       </c>
       <c r="M3" t="n">
-        <v>0.0798278847555796</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0.458211176424905</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0.525355029574027</v>
-      </c>
-      <c r="P3" t="e">
-        <v>#NUM!</v>
-      </c>
-      <c r="Q3" t="e">
-        <v>#NUM!</v>
+        <v>0.496825302686603</v>
+      </c>
+      <c r="N3" t="e">
+        <v>#NUM!</v>
+      </c>
+      <c r="O3" t="e">
+        <v>#NUM!</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.30711256121321</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0.386474765493542</v>
       </c>
       <c r="R3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S3" t="n">
-        <v>0</v>
-      </c>
-      <c r="T3" t="n">
-        <v>1</v>
+        <v>0.306412673293248</v>
       </c>
     </row>
     <row r="4">
@@ -591,61 +567,55 @@
         <v>4</v>
       </c>
       <c r="B4" t="n">
-        <v>1775</v>
+        <v>1110</v>
       </c>
       <c r="C4" t="n">
-        <v>3.87380281690141</v>
+        <v>3.08018018018018</v>
       </c>
       <c r="D4" t="n">
-        <v>10235.3135211268</v>
+        <v>8290.09018018018</v>
       </c>
       <c r="E4" t="n">
-        <v>4654.91678873239</v>
+        <v>3758.06927927928</v>
       </c>
       <c r="F4" t="n">
-        <v>166.367323943662</v>
+        <v>202.838738738739</v>
       </c>
       <c r="G4" t="n">
-        <v>2.92619718309859</v>
+        <v>2.68468468468468</v>
       </c>
       <c r="H4" t="n">
-        <v>1190.51236243895</v>
-      </c>
-      <c r="I4" t="e">
-        <v>#NUM!</v>
+        <v>1233.77575602742</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.75517014303779</v>
       </c>
       <c r="J4" t="n">
-        <v>0.280303960256909</v>
+        <v>0.0428705349808459</v>
       </c>
       <c r="K4" t="n">
-        <v>0.177464788732394</v>
+        <v>0.0730312408255343</v>
       </c>
       <c r="L4" t="n">
-        <v>0.0478028025663003</v>
+        <v>0.45171541615728</v>
       </c>
       <c r="M4" t="n">
-        <v>0.0795584699544066</v>
-      </c>
-      <c r="N4" t="n">
-        <v>0.450096717109285</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0.453199082031109</v>
-      </c>
-      <c r="P4" t="e">
-        <v>#NUM!</v>
-      </c>
-      <c r="Q4" t="e">
-        <v>#NUM!</v>
+        <v>0.537162775545128</v>
+      </c>
+      <c r="N4" t="e">
+        <v>#NUM!</v>
+      </c>
+      <c r="O4" t="e">
+        <v>#NUM!</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.304701985731398</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.407696558578912</v>
       </c>
       <c r="R4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S4" t="n">
-        <v>1</v>
-      </c>
-      <c r="T4" t="n">
-        <v>0</v>
+        <v>0.287601455689691</v>
       </c>
     </row>
     <row r="5">
@@ -653,123 +623,111 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>1760</v>
+        <v>1690</v>
       </c>
       <c r="C5" t="n">
-        <v>1.85454545454545</v>
+        <v>2.01420118343195</v>
       </c>
       <c r="D5" t="n">
-        <v>4311.96573863636</v>
+        <v>4752.39195266272</v>
       </c>
       <c r="E5" t="n">
-        <v>2023.74909090909</v>
+        <v>2223.23905325444</v>
       </c>
       <c r="F5" t="n">
-        <v>282.673863636364</v>
+        <v>268.820118343195</v>
       </c>
       <c r="G5" t="n">
-        <v>1.68579545454545</v>
+        <v>1.67100591715976</v>
       </c>
       <c r="H5" t="n">
-        <v>1331.75096336129</v>
-      </c>
-      <c r="I5" t="e">
-        <v>#NUM!</v>
+        <v>1346.42503483055</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.177666158627697</v>
       </c>
       <c r="J5" t="n">
-        <v>0.289352904040404</v>
+        <v>0.0212518653273091</v>
       </c>
       <c r="K5" t="n">
-        <v>0.243181818181818</v>
+        <v>0.0375368634953332</v>
       </c>
       <c r="L5" t="n">
-        <v>0.0181136887102796</v>
+        <v>0.470320139422764</v>
       </c>
       <c r="M5" t="n">
-        <v>0.0325485804183364</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0.472658796281896</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0.751183937590188</v>
-      </c>
-      <c r="P5" t="e">
-        <v>#NUM!</v>
-      </c>
-      <c r="Q5" t="e">
-        <v>#NUM!</v>
+        <v>0.7587097304405</v>
+      </c>
+      <c r="N5" t="e">
+        <v>#NUM!</v>
+      </c>
+      <c r="O5" t="e">
+        <v>#NUM!</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.254074621959237</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.51041678407063</v>
       </c>
       <c r="R5" t="n">
-        <v>0.557954545454545</v>
-      </c>
-      <c r="S5" t="n">
-        <v>0.316477272727273</v>
-      </c>
-      <c r="T5" t="n">
-        <v>0.125568181818182</v>
+        <v>0.235508593970132</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B6" t="n">
-        <v>454</v>
+        <v>372</v>
       </c>
       <c r="C6" t="n">
-        <v>2.33259911894273</v>
+        <v>2.25537634408602</v>
       </c>
       <c r="D6" t="n">
-        <v>2872.58215859031</v>
+        <v>2489.6997311828</v>
       </c>
       <c r="E6" t="n">
-        <v>-65.538986784141</v>
+        <v>-238.896505376344</v>
       </c>
       <c r="F6" t="n">
-        <v>235.988986784141</v>
+        <v>244.389784946237</v>
       </c>
       <c r="G6" t="n">
-        <v>2.23568281938326</v>
+        <v>2.15591397849462</v>
       </c>
       <c r="H6" t="n">
-        <v>587.764305929631</v>
-      </c>
-      <c r="I6" t="e">
-        <v>#NUM!</v>
+        <v>536.050982005599</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.277549004161907</v>
       </c>
       <c r="J6" t="n">
-        <v>0.297156697927623</v>
+        <v>0.304438029193971</v>
       </c>
       <c r="K6" t="n">
-        <v>0.237885462555066</v>
+        <v>0.571253095059525</v>
       </c>
       <c r="L6" t="n">
-        <v>0.284536708200035</v>
+        <v>-0.189291273518763</v>
       </c>
       <c r="M6" t="n">
-        <v>0.529990605074082</v>
-      </c>
-      <c r="N6" t="n">
-        <v>-0.121207133757805</v>
-      </c>
-      <c r="O6" t="n">
-        <v>0.620598845598846</v>
-      </c>
-      <c r="P6" t="e">
-        <v>#NUM!</v>
-      </c>
-      <c r="Q6" t="e">
-        <v>#NUM!</v>
+        <v>0.632603186837058</v>
+      </c>
+      <c r="N6" t="e">
+        <v>#NUM!</v>
+      </c>
+      <c r="O6" t="e">
+        <v>#NUM!</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0.301297716620297</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0.409460439500762</v>
       </c>
       <c r="R6" t="n">
-        <v>0.491189427312775</v>
-      </c>
-      <c r="S6" t="n">
-        <v>0.383259911894273</v>
-      </c>
-      <c r="T6" t="n">
-        <v>0.125550660792952</v>
+        <v>0.289241843878941</v>
       </c>
     </row>
   </sheetData>

</xml_diff>